<commit_message>
auto: session 2026-10-27 15:10
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/11-bao-gia-khach/Bao-Gia-PR-Hoa-Hoc-Tro-Webtretho-2026-10-27.xlsx
+++ b/11-bao-gia-khach/Bao-Gia-PR-Hoa-Hoc-Tro-Webtretho-2026-10-27.xlsx
@@ -752,7 +752,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Bài PR theo nội dung khách hàng cung cấp. Bên bán hỗ trợ biên tập bài để khách duyệt trước khi gửi toà soạn (phí viết bài mới tính riêng nếu có).</t>
+          <t>Bài PR theo nội dung khách hàng cung cấp. Giá đã bao gồm phí viết bài và biên tập; bên bán gửi bài để khách duyệt trước khi gửi toà soạn.</t>
         </is>
       </c>
     </row>
@@ -1051,10 +1051,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A17:B17"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A17:B17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>